<commit_message>
add a new true false column in excel
</commit_message>
<xml_diff>
--- a/testing-folder/tcg_data_categoryId86.xlsx
+++ b/testing-folder/tcg_data_categoryId86.xlsx
@@ -575,7 +575,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/710638_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/710638_400w.jpg</t>
         </is>
       </c>
       <c r="K2" t="n">
@@ -602,10 +602,20 @@
           <t>2026-09-25T00:00:00</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="R2" t="n">
+        <v>37.99</v>
+      </c>
+      <c r="S2" t="n">
+        <v>37.99</v>
+      </c>
+      <c r="T2" t="n">
+        <v>37.99</v>
+      </c>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="b">
@@ -654,7 +664,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/710640_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/710640_400w.jpg</t>
         </is>
       </c>
       <c r="K3" t="n">
@@ -697,7 +707,9 @@
       </c>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
+      <c r="W3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -741,7 +753,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/710641_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/710641_400w.jpg</t>
         </is>
       </c>
       <c r="K4" t="n">
@@ -820,7 +832,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/662118_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/662118_400w.jpg</t>
         </is>
       </c>
       <c r="K5" t="n">
@@ -856,16 +868,18 @@
         <v>17.27</v>
       </c>
       <c r="S5" t="n">
-        <v>21.14</v>
+        <v>22</v>
       </c>
       <c r="T5" t="n">
         <v>129.99</v>
       </c>
       <c r="U5" t="n">
-        <v>20.06</v>
+        <v>19.76</v>
       </c>
       <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
+      <c r="W5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -909,7 +923,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/662119_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/662119_400w.jpg</t>
         </is>
       </c>
       <c r="K6" t="n">
@@ -945,16 +959,18 @@
         <v>74.84999999999999</v>
       </c>
       <c r="S6" t="n">
-        <v>78.94</v>
+        <v>78.95</v>
       </c>
       <c r="T6" t="n">
         <v>119.74</v>
       </c>
       <c r="U6" t="n">
-        <v>75.18000000000001</v>
+        <v>74.88</v>
       </c>
       <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
+      <c r="W6" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -998,7 +1014,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/662120_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/662120_400w.jpg</t>
         </is>
       </c>
       <c r="K7" t="n">
@@ -1077,7 +1093,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/670551_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/670551_400w.jpg</t>
         </is>
       </c>
       <c r="K8" t="n">
@@ -1113,16 +1129,18 @@
         <v>0.25</v>
       </c>
       <c r="S8" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="T8" t="n">
         <v>99.90000000000001</v>
       </c>
       <c r="U8" t="n">
-        <v>0.53</v>
+        <v>0.52</v>
       </c>
       <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
+      <c r="W8" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1166,7 +1184,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/670552_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/670552_400w.jpg</t>
         </is>
       </c>
       <c r="K9" t="n">
@@ -1211,7 +1229,9 @@
         <v>0.12</v>
       </c>
       <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
+      <c r="W9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1255,7 +1275,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/670553_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/670553_400w.jpg</t>
         </is>
       </c>
       <c r="K10" t="n">
@@ -1300,7 +1320,9 @@
         <v>0.12</v>
       </c>
       <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
+      <c r="W10" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1344,7 +1366,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/670554_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/670554_400w.jpg</t>
         </is>
       </c>
       <c r="K11" t="n">
@@ -1389,7 +1411,9 @@
         <v>0.12</v>
       </c>
       <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
+      <c r="W11" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1433,7 +1457,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/670555_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/670555_400w.jpg</t>
         </is>
       </c>
       <c r="K12" t="n">
@@ -1469,16 +1493,18 @@
         <v>0.15</v>
       </c>
       <c r="S12" t="n">
-        <v>0.32</v>
+        <v>0.35</v>
       </c>
       <c r="T12" t="n">
         <v>3</v>
       </c>
       <c r="U12" t="n">
-        <v>0.31</v>
+        <v>0.33</v>
       </c>
       <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
+      <c r="W12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1522,7 +1548,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/670556_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/670556_400w.jpg</t>
         </is>
       </c>
       <c r="K13" t="n">
@@ -1567,7 +1593,9 @@
         <v>0.14</v>
       </c>
       <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
+      <c r="W13" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1611,7 +1639,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/670557_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/670557_400w.jpg</t>
         </is>
       </c>
       <c r="K14" t="n">
@@ -1656,7 +1684,9 @@
         <v>0.12</v>
       </c>
       <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
+      <c r="W14" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1700,7 +1730,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/670558_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/670558_400w.jpg</t>
         </is>
       </c>
       <c r="K15" t="n">
@@ -1741,7 +1771,9 @@
         <v>0.19</v>
       </c>
       <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
+      <c r="W15" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1785,7 +1817,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/670559_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/670559_400w.jpg</t>
         </is>
       </c>
       <c r="K16" t="n">
@@ -1830,7 +1862,9 @@
         <v>0.13</v>
       </c>
       <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
+      <c r="W16" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1874,7 +1908,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/670560_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/670560_400w.jpg</t>
         </is>
       </c>
       <c r="K17" t="n">
@@ -1919,7 +1953,9 @@
         <v>0.13</v>
       </c>
       <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
+      <c r="W17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1963,7 +1999,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/670561_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/670561_400w.jpg</t>
         </is>
       </c>
       <c r="K18" t="n">
@@ -1999,7 +2035,7 @@
         <v>1.49</v>
       </c>
       <c r="S18" t="n">
-        <v>1.99</v>
+        <v>1.98</v>
       </c>
       <c r="T18" t="n">
         <v>9.99</v>
@@ -2008,7 +2044,9 @@
         <v>1.75</v>
       </c>
       <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
+      <c r="W18" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2052,7 +2090,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671948_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671948_400w.jpg</t>
         </is>
       </c>
       <c r="K19" t="n">
@@ -2097,7 +2135,9 @@
         <v>0.24</v>
       </c>
       <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
+      <c r="W19" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -2141,7 +2181,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671951_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671951_400w.jpg</t>
         </is>
       </c>
       <c r="K20" t="n">
@@ -2183,10 +2223,12 @@
         <v>99.90000000000001</v>
       </c>
       <c r="U20" t="n">
-        <v>0.55</v>
+        <v>0.54</v>
       </c>
       <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr"/>
+      <c r="W20" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2230,7 +2272,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671956_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671956_400w.jpg</t>
         </is>
       </c>
       <c r="K21" t="n">
@@ -2275,7 +2317,9 @@
         <v>0.15</v>
       </c>
       <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
+      <c r="W21" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2319,7 +2363,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671960_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671960_400w.jpg</t>
         </is>
       </c>
       <c r="K22" t="n">
@@ -2364,7 +2408,9 @@
         <v>0.23</v>
       </c>
       <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr"/>
+      <c r="W22" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2408,7 +2454,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671963_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671963_400w.jpg</t>
         </is>
       </c>
       <c r="K23" t="n">
@@ -2453,7 +2499,9 @@
         <v>0.11</v>
       </c>
       <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
+      <c r="W23" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2497,7 +2545,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671968_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671968_400w.jpg</t>
         </is>
       </c>
       <c r="K24" t="n">
@@ -2526,7 +2574,7 @@
         </is>
       </c>
       <c r="R24" t="n">
-        <v>36</v>
+        <v>40.89</v>
       </c>
       <c r="S24" t="n">
         <v>45</v>
@@ -2535,10 +2583,12 @@
         <v>48.91</v>
       </c>
       <c r="U24" t="n">
-        <v>41.62</v>
+        <v>41.77</v>
       </c>
       <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
+      <c r="W24" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2582,7 +2632,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671969_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671969_400w.jpg</t>
         </is>
       </c>
       <c r="K25" t="n">
@@ -2614,7 +2664,7 @@
         <v>8.51</v>
       </c>
       <c r="S25" t="n">
-        <v>14.5</v>
+        <v>13</v>
       </c>
       <c r="T25" t="n">
         <v>99.90000000000001</v>
@@ -2623,7 +2673,9 @@
         <v>10.68</v>
       </c>
       <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
+      <c r="W25" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2667,7 +2719,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671970_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671970_400w.jpg</t>
         </is>
       </c>
       <c r="K26" t="n">
@@ -2696,7 +2748,7 @@
         </is>
       </c>
       <c r="R26" t="n">
-        <v>3</v>
+        <v>2.99</v>
       </c>
       <c r="S26" t="n">
         <v>3.54</v>
@@ -2708,7 +2760,9 @@
         <v>3.47</v>
       </c>
       <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr"/>
+      <c r="W26" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2752,7 +2806,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671971_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671971_400w.jpg</t>
         </is>
       </c>
       <c r="K27" t="n">
@@ -2781,7 +2835,7 @@
         </is>
       </c>
       <c r="R27" t="n">
-        <v>3</v>
+        <v>2.99</v>
       </c>
       <c r="S27" t="n">
         <v>4.58</v>
@@ -2793,7 +2847,9 @@
         <v>4.17</v>
       </c>
       <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
+      <c r="W27" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2837,7 +2893,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671972_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671972_400w.jpg</t>
         </is>
       </c>
       <c r="K28" t="n">
@@ -2866,19 +2922,21 @@
         </is>
       </c>
       <c r="R28" t="n">
-        <v>16.5</v>
+        <v>16</v>
       </c>
       <c r="S28" t="n">
-        <v>23.53</v>
+        <v>23.9</v>
       </c>
       <c r="T28" t="n">
         <v>99.90000000000001</v>
       </c>
       <c r="U28" t="n">
-        <v>22.85</v>
+        <v>22.55</v>
       </c>
       <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
+      <c r="W28" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2922,7 +2980,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671973_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671973_400w.jpg</t>
         </is>
       </c>
       <c r="K29" t="n">
@@ -2954,7 +3012,7 @@
         <v>1.5</v>
       </c>
       <c r="S29" t="n">
-        <v>3.77</v>
+        <v>3.59</v>
       </c>
       <c r="T29" t="n">
         <v>25</v>
@@ -2963,7 +3021,9 @@
         <v>2.67</v>
       </c>
       <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr"/>
+      <c r="W29" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -3007,7 +3067,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671974_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671974_400w.jpg</t>
         </is>
       </c>
       <c r="K30" t="n">
@@ -3048,7 +3108,9 @@
         <v>1.69</v>
       </c>
       <c r="V30" t="inlineStr"/>
-      <c r="W30" t="inlineStr"/>
+      <c r="W30" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -3092,7 +3154,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671975_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671975_400w.jpg</t>
         </is>
       </c>
       <c r="K31" t="n">
@@ -3124,7 +3186,7 @@
         <v>12</v>
       </c>
       <c r="S31" t="n">
-        <v>15.56</v>
+        <v>15</v>
       </c>
       <c r="T31" t="n">
         <v>99.90000000000001</v>
@@ -3133,7 +3195,9 @@
         <v>10.97</v>
       </c>
       <c r="V31" t="inlineStr"/>
-      <c r="W31" t="inlineStr"/>
+      <c r="W31" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -3177,7 +3241,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671976_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671976_400w.jpg</t>
         </is>
       </c>
       <c r="K32" t="n">
@@ -3209,7 +3273,7 @@
         <v>30.03</v>
       </c>
       <c r="S32" t="n">
-        <v>91</v>
+        <v>50</v>
       </c>
       <c r="T32" t="n">
         <v>99.90000000000001</v>
@@ -3218,7 +3282,9 @@
         <v>33.27</v>
       </c>
       <c r="V32" t="inlineStr"/>
-      <c r="W32" t="inlineStr"/>
+      <c r="W32" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -3262,7 +3328,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671977_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671977_400w.jpg</t>
         </is>
       </c>
       <c r="K33" t="n">
@@ -3291,7 +3357,7 @@
         </is>
       </c>
       <c r="R33" t="n">
-        <v>7.5</v>
+        <v>5.41</v>
       </c>
       <c r="S33" t="n">
         <v>9.02</v>
@@ -3303,7 +3369,9 @@
         <v>7.27</v>
       </c>
       <c r="V33" t="inlineStr"/>
-      <c r="W33" t="inlineStr"/>
+      <c r="W33" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -3347,7 +3415,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671978_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671978_400w.jpg</t>
         </is>
       </c>
       <c r="K34" t="n">
@@ -3376,10 +3444,10 @@
         </is>
       </c>
       <c r="R34" t="n">
-        <v>16.5</v>
+        <v>15.57</v>
       </c>
       <c r="S34" t="n">
-        <v>20.03</v>
+        <v>18.34</v>
       </c>
       <c r="T34" t="n">
         <v>74.98999999999999</v>
@@ -3388,7 +3456,9 @@
         <v>17.96</v>
       </c>
       <c r="V34" t="inlineStr"/>
-      <c r="W34" t="inlineStr"/>
+      <c r="W34" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -3432,7 +3502,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671979_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671979_400w.jpg</t>
         </is>
       </c>
       <c r="K35" t="n">
@@ -3464,16 +3534,18 @@
         <v>5</v>
       </c>
       <c r="S35" t="n">
-        <v>8</v>
+        <v>7.99</v>
       </c>
       <c r="T35" t="n">
         <v>10.99</v>
       </c>
       <c r="U35" t="n">
-        <v>7.18</v>
+        <v>7.22</v>
       </c>
       <c r="V35" t="inlineStr"/>
-      <c r="W35" t="inlineStr"/>
+      <c r="W35" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -3517,7 +3589,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671980_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671980_400w.jpg</t>
         </is>
       </c>
       <c r="K36" t="n">
@@ -3549,16 +3621,18 @@
         <v>49.99</v>
       </c>
       <c r="S36" t="n">
-        <v>50</v>
+        <v>52.5</v>
       </c>
       <c r="T36" t="n">
         <v>79.98999999999999</v>
       </c>
       <c r="U36" t="n">
-        <v>40.57</v>
+        <v>41.04</v>
       </c>
       <c r="V36" t="inlineStr"/>
-      <c r="W36" t="inlineStr"/>
+      <c r="W36" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -3602,7 +3676,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671981_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671981_400w.jpg</t>
         </is>
       </c>
       <c r="K37" t="n">
@@ -3634,16 +3708,18 @@
         <v>5</v>
       </c>
       <c r="S37" t="n">
-        <v>6.03</v>
+        <v>6.07</v>
       </c>
       <c r="T37" t="n">
         <v>23.99</v>
       </c>
       <c r="U37" t="n">
-        <v>5.23</v>
+        <v>5.3</v>
       </c>
       <c r="V37" t="inlineStr"/>
-      <c r="W37" t="inlineStr"/>
+      <c r="W37" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -3687,7 +3763,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671982_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671982_400w.jpg</t>
         </is>
       </c>
       <c r="K38" t="n">
@@ -3725,10 +3801,12 @@
         <v>40</v>
       </c>
       <c r="U38" t="n">
-        <v>13.3</v>
+        <v>13.22</v>
       </c>
       <c r="V38" t="inlineStr"/>
-      <c r="W38" t="inlineStr"/>
+      <c r="W38" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -3772,7 +3850,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/671983_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/671983_400w.jpg</t>
         </is>
       </c>
       <c r="K39" t="n">
@@ -3804,7 +3882,7 @@
         <v>0.99</v>
       </c>
       <c r="S39" t="n">
-        <v>2.25</v>
+        <v>2</v>
       </c>
       <c r="T39" t="n">
         <v>15</v>
@@ -3813,7 +3891,9 @@
         <v>1.36</v>
       </c>
       <c r="V39" t="inlineStr"/>
-      <c r="W39" t="inlineStr"/>
+      <c r="W39" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -3857,7 +3937,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>https://tcgplayer-cdn.tcgplayer.com/product/672971_200w.jpg</t>
+          <t>https://tcgplayer-cdn.tcgplayer.com/product/672971_400w.jpg</t>
         </is>
       </c>
       <c r="K40" t="n">

</xml_diff>